<commit_message>
Momentum scan results 2026-08-23
</commit_message>
<xml_diff>
--- a/results/momentum_merged_latest.xlsx
+++ b/results/momentum_merged_latest.xlsx
@@ -903,7 +903,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>ASST</t>
+          <t>ASPCU</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -925,7 +925,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>ATLO</t>
+          <t>ASST</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -947,7 +947,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>AU</t>
+          <t>ATLO</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -969,7 +969,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>AUGO</t>
+          <t>AU</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -991,7 +991,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>AXGN</t>
+          <t>AUGO</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1013,22 +1013,22 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
+          <t>AXGN</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>AREC</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>OCG</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
           <t>AXIN</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>AREC</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>OCG</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>AYTU</t>
         </is>
       </c>
     </row>
@@ -1045,7 +1045,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>AZTA</t>
+          <t>AYTU</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -1062,7 +1062,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>BANFP</t>
+          <t>AZTA</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1079,22 +1079,22 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
+          <t>BANFP</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>ATRA</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>PUSA</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
           <t>BCPC</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>ATRA</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>PUSA</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>BCTX</t>
         </is>
       </c>
     </row>
@@ -1111,7 +1111,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>BDSX</t>
+          <t>BCTX</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -1128,7 +1128,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>BDTX</t>
+          <t>BDSX</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1145,22 +1145,22 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
+          <t>BDTX</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>AVO</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>SOUN</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
           <t>BEEM</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>AVO</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>SOUN</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>BLFS</t>
         </is>
       </c>
     </row>
@@ -1177,7 +1177,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>BLMN</t>
+          <t>BLFS</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -1194,17 +1194,17 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
+          <t>BLMN</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>AVTR</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
           <t>BLSH</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>AVTR</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>BMNP</t>
         </is>
       </c>
     </row>
@@ -1216,17 +1216,17 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
+          <t>BMNP</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>BCDA</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
           <t>BMNR</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>BCDA</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>BNTX</t>
         </is>
       </c>
     </row>
@@ -1238,17 +1238,17 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
+          <t>BNTX</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>BETA</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
           <t>BPYPP</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>BETA</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>BRNX</t>
         </is>
       </c>
     </row>
@@ -1260,17 +1260,17 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
+          <t>BRNX</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>BLKB</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
           <t>BRZE</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>BLKB</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>BTBD</t>
         </is>
       </c>
     </row>
@@ -1282,17 +1282,17 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
+          <t>BTBD</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>BOLD</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
           <t>BTCS</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>BOLD</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>BTGO</t>
         </is>
       </c>
     </row>
@@ -1304,17 +1304,17 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
+          <t>BTGO</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>BPYPO</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
           <t>BULLW</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>BPYPO</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>BWB</t>
         </is>
       </c>
     </row>
@@ -1326,17 +1326,17 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
+          <t>BWB</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>BRCB</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
           <t>CAI</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>BRCB</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>CCSI</t>
         </is>
       </c>
     </row>
@@ -1348,17 +1348,17 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
+          <t>CCSI</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>BSY</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
           <t>CDLR</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>BSY</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>CDNA</t>
         </is>
       </c>
     </row>
@@ -1370,17 +1370,17 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
+          <t>CDNA</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>BVC</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
           <t>CEPO</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>BVC</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>CGAU</t>
         </is>
       </c>
     </row>
@@ -1392,17 +1392,17 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
+          <t>CGAU</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>BYND</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
           <t>CHDN</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>BYND</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>CHTRP</t>
         </is>
       </c>
     </row>
@@ -1414,17 +1414,17 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
+          <t>CHTRP</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>CCC</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
           <t>CING</t>
-        </is>
-      </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>CCC</t>
-        </is>
-      </c>
-      <c r="D46" t="inlineStr">
-        <is>
-          <t>CITR</t>
         </is>
       </c>
     </row>
@@ -1436,17 +1436,17 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
+          <t>CITR</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>CCG</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
           <t>CME</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>CCG</t>
-        </is>
-      </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>CMMB</t>
         </is>
       </c>
     </row>
@@ -1458,17 +1458,17 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
+          <t>CMMB</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>CELU</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
           <t>CMTV</t>
-        </is>
-      </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>CELU</t>
-        </is>
-      </c>
-      <c r="D48" t="inlineStr">
-        <is>
-          <t>CNOBP</t>
         </is>
       </c>
     </row>
@@ -1480,17 +1480,17 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
+          <t>CNOBP</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>CHCI</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
           <t>CNR</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>CHCI</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>COCP</t>
         </is>
       </c>
     </row>
@@ -1502,17 +1502,17 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
+          <t>COCP</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>CLBK</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
           <t>CRBP</t>
-        </is>
-      </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>CLBK</t>
-        </is>
-      </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>CSHR</t>
         </is>
       </c>
     </row>
@@ -1524,17 +1524,17 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
+          <t>CSHR</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>CMPS</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
           <t>CSTL</t>
-        </is>
-      </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>CMPS</t>
-        </is>
-      </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>CSX</t>
         </is>
       </c>
     </row>
@@ -1546,17 +1546,17 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
+          <t>CSX</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>COKE</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
           <t>CTRM</t>
-        </is>
-      </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>COKE</t>
-        </is>
-      </c>
-      <c r="D52" t="inlineStr">
-        <is>
-          <t>CVSA</t>
         </is>
       </c>
     </row>
@@ -1568,17 +1568,17 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
+          <t>CVSA</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>CPB</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
           <t>CYCN</t>
-        </is>
-      </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>CPB</t>
-        </is>
-      </c>
-      <c r="D53" t="inlineStr">
-        <is>
-          <t>CYPH</t>
         </is>
       </c>
     </row>
@@ -1590,17 +1590,17 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
+          <t>CYPH</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>CRMD</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
           <t>CYRX</t>
-        </is>
-      </c>
-      <c r="C54" t="inlineStr">
-        <is>
-          <t>CRMD</t>
-        </is>
-      </c>
-      <c r="D54" t="inlineStr">
-        <is>
-          <t>CZFS</t>
         </is>
       </c>
     </row>
@@ -1612,17 +1612,17 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
+          <t>CZFS</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>CRVL</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
           <t>DCBO</t>
-        </is>
-      </c>
-      <c r="C55" t="inlineStr">
-        <is>
-          <t>CRVL</t>
-        </is>
-      </c>
-      <c r="D55" t="inlineStr">
-        <is>
-          <t>DCH</t>
         </is>
       </c>
     </row>
@@ -1634,17 +1634,17 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
+          <t>DCH</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>CSWC</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
           <t>DDI</t>
-        </is>
-      </c>
-      <c r="C56" t="inlineStr">
-        <is>
-          <t>CSWC</t>
-        </is>
-      </c>
-      <c r="D56" t="inlineStr">
-        <is>
-          <t>DFDV</t>
         </is>
       </c>
     </row>
@@ -1656,17 +1656,17 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
+          <t>DFDV</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>CTSH</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
           <t>DHCNI</t>
-        </is>
-      </c>
-      <c r="C57" t="inlineStr">
-        <is>
-          <t>CTSH</t>
-        </is>
-      </c>
-      <c r="D57" t="inlineStr">
-        <is>
-          <t>DMAA</t>
         </is>
       </c>
     </row>
@@ -1678,17 +1678,17 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
+          <t>DMAA</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>CZNC</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
           <t>DMLP</t>
-        </is>
-      </c>
-      <c r="C58" t="inlineStr">
-        <is>
-          <t>CZNC</t>
-        </is>
-      </c>
-      <c r="D58" t="inlineStr">
-        <is>
-          <t>DOX</t>
         </is>
       </c>
     </row>
@@ -1700,17 +1700,17 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
+          <t>DOX</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>DASH</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
           <t>DRTS</t>
-        </is>
-      </c>
-      <c r="C59" t="inlineStr">
-        <is>
-          <t>DASH</t>
-        </is>
-      </c>
-      <c r="D59" t="inlineStr">
-        <is>
-          <t>DRUG</t>
         </is>
       </c>
     </row>
@@ -1722,17 +1722,17 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
+          <t>DRUG</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>DERM</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
           <t>DSGN</t>
-        </is>
-      </c>
-      <c r="C60" t="inlineStr">
-        <is>
-          <t>DERM</t>
-        </is>
-      </c>
-      <c r="D60" t="inlineStr">
-        <is>
-          <t>DTCX</t>
         </is>
       </c>
     </row>
@@ -1744,17 +1744,17 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
+          <t>DTCX</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>DKNG</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
           <t>DTIL</t>
-        </is>
-      </c>
-      <c r="C61" t="inlineStr">
-        <is>
-          <t>DKNG</t>
-        </is>
-      </c>
-      <c r="D61" t="inlineStr">
-        <is>
-          <t>DWTX</t>
         </is>
       </c>
     </row>
@@ -1766,17 +1766,17 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
+          <t>DWTX</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>DSC</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
           <t>EDRY</t>
-        </is>
-      </c>
-      <c r="C62" t="inlineStr">
-        <is>
-          <t>DSC</t>
-        </is>
-      </c>
-      <c r="D62" t="inlineStr">
-        <is>
-          <t>ELBM</t>
         </is>
       </c>
     </row>
@@ -1788,17 +1788,17 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
+          <t>ELBM</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>DXCM</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
           <t>ELLA</t>
-        </is>
-      </c>
-      <c r="C63" t="inlineStr">
-        <is>
-          <t>DXCM</t>
-        </is>
-      </c>
-      <c r="D63" t="inlineStr">
-        <is>
-          <t>ELMT</t>
         </is>
       </c>
     </row>
@@ -1810,17 +1810,17 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
+          <t>ELMT</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>EFOR</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
           <t>ELOX</t>
-        </is>
-      </c>
-      <c r="C64" t="inlineStr">
-        <is>
-          <t>EFOR</t>
-        </is>
-      </c>
-      <c r="D64" t="inlineStr">
-        <is>
-          <t>ENTX</t>
         </is>
       </c>
     </row>
@@ -1832,17 +1832,17 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
+          <t>ENTX</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>ELE</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
           <t>EPRX</t>
-        </is>
-      </c>
-      <c r="C65" t="inlineStr">
-        <is>
-          <t>ELE</t>
-        </is>
-      </c>
-      <c r="D65" t="inlineStr">
-        <is>
-          <t>EXE</t>
         </is>
       </c>
     </row>
@@ -1854,17 +1854,17 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
+          <t>EXE</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>EROK</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
           <t>EXPE</t>
-        </is>
-      </c>
-      <c r="C66" t="inlineStr">
-        <is>
-          <t>EROK</t>
-        </is>
-      </c>
-      <c r="D66" t="inlineStr">
-        <is>
-          <t>EXPO</t>
         </is>
       </c>
     </row>
@@ -1876,17 +1876,17 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
+          <t>EXPO</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>EXFY</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
           <t>FBLG</t>
-        </is>
-      </c>
-      <c r="C67" t="inlineStr">
-        <is>
-          <t>EXFY</t>
-        </is>
-      </c>
-      <c r="D67" t="inlineStr">
-        <is>
-          <t>FBRX</t>
         </is>
       </c>
     </row>
@@ -1898,17 +1898,17 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
+          <t>FBRX</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>FCBC</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
           <t>FHTX</t>
-        </is>
-      </c>
-      <c r="C68" t="inlineStr">
-        <is>
-          <t>FCBC</t>
-        </is>
-      </c>
-      <c r="D68" t="inlineStr">
-        <is>
-          <t>FIVE</t>
         </is>
       </c>
     </row>
@@ -1920,17 +1920,17 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
+          <t>FIVE</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>FEAM</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
           <t>FIZZ</t>
-        </is>
-      </c>
-      <c r="C69" t="inlineStr">
-        <is>
-          <t>FEAM</t>
-        </is>
-      </c>
-      <c r="D69" t="inlineStr">
-        <is>
-          <t>FLNT</t>
         </is>
       </c>
     </row>
@@ -1942,17 +1942,17 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
+          <t>FLNT</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>FERA</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
           <t>FLYW</t>
-        </is>
-      </c>
-      <c r="C70" t="inlineStr">
-        <is>
-          <t>FERA</t>
-        </is>
-      </c>
-      <c r="D70" t="inlineStr">
-        <is>
-          <t>FRHC</t>
         </is>
       </c>
     </row>
@@ -1964,17 +1964,17 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
+          <t>FRHC</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>FIVN</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
           <t>FTDR</t>
-        </is>
-      </c>
-      <c r="C71" t="inlineStr">
-        <is>
-          <t>FIVN</t>
-        </is>
-      </c>
-      <c r="D71" t="inlineStr">
-        <is>
-          <t>FTH</t>
         </is>
       </c>
     </row>
@@ -1986,17 +1986,17 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
+          <t>FTH</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>FNKO</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
           <t>FUTU</t>
-        </is>
-      </c>
-      <c r="C72" t="inlineStr">
-        <is>
-          <t>FNKO</t>
-        </is>
-      </c>
-      <c r="D72" t="inlineStr">
-        <is>
-          <t>FVN</t>
         </is>
       </c>
     </row>
@@ -2008,17 +2008,17 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
+          <t>FVN</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>FOX</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
           <t>FWDI</t>
-        </is>
-      </c>
-      <c r="C73" t="inlineStr">
-        <is>
-          <t>FOX</t>
-        </is>
-      </c>
-      <c r="D73" t="inlineStr">
-        <is>
-          <t>GAINZ</t>
         </is>
       </c>
     </row>
@@ -2030,17 +2030,17 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
+          <t>GAINZ</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>FRNM</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
           <t>GECCI</t>
-        </is>
-      </c>
-      <c r="C74" t="inlineStr">
-        <is>
-          <t>FRNM</t>
-        </is>
-      </c>
-      <c r="D74" t="inlineStr">
-        <is>
-          <t>GIBO</t>
         </is>
       </c>
     </row>
@@ -2052,17 +2052,17 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
+          <t>GIBO</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>FWONA</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
           <t>GOLD</t>
-        </is>
-      </c>
-      <c r="C75" t="inlineStr">
-        <is>
-          <t>FWONA</t>
-        </is>
-      </c>
-      <c r="D75" t="inlineStr">
-        <is>
-          <t>GYRE</t>
         </is>
       </c>
     </row>
@@ -2074,1327 +2074,1327 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
+          <t>GYRE</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>GCBC</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
           <t>HAIN</t>
-        </is>
-      </c>
-      <c r="C76" t="inlineStr">
-        <is>
-          <t>GAME</t>
-        </is>
-      </c>
-      <c r="D76" t="inlineStr">
-        <is>
-          <t>HELP</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>GCBC</t>
+          <t>GDYN</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
+          <t>HELP</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>GECCG</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
           <t>HLXC</t>
-        </is>
-      </c>
-      <c r="C77" t="inlineStr">
-        <is>
-          <t>GDYN</t>
-        </is>
-      </c>
-      <c r="D77" t="inlineStr">
-        <is>
-          <t>HOLO</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>GECCG</t>
+          <t>GEHC</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
+          <t>HOLO</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>GH</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
           <t>HQI</t>
-        </is>
-      </c>
-      <c r="C78" t="inlineStr">
-        <is>
-          <t>GEHC</t>
-        </is>
-      </c>
-      <c r="D78" t="inlineStr">
-        <is>
-          <t>HYNE</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>GH</t>
+          <t>GLBS</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
+          <t>HYNE</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>GMRS</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
           <t>HYPD</t>
-        </is>
-      </c>
-      <c r="C79" t="inlineStr">
-        <is>
-          <t>GLBS</t>
-        </is>
-      </c>
-      <c r="D79" t="inlineStr">
-        <is>
-          <t>IBKR</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>GMRS</t>
+          <t>GO</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
+          <t>IBKR</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>GP</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
           <t>IDYA</t>
-        </is>
-      </c>
-      <c r="C80" t="inlineStr">
-        <is>
-          <t>GO</t>
-        </is>
-      </c>
-      <c r="D80" t="inlineStr">
-        <is>
-          <t>ILMN</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>GP</t>
+          <t>GRAL</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
+          <t>ILMN</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>GROW</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
           <t>IMPP</t>
-        </is>
-      </c>
-      <c r="C81" t="inlineStr">
-        <is>
-          <t>GRAL</t>
-        </is>
-      </c>
-      <c r="D81" t="inlineStr">
-        <is>
-          <t>INFQ</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>GROW</t>
+          <t>GRRR</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
+          <t>INFQ</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>GRVY</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
           <t>INMB</t>
-        </is>
-      </c>
-      <c r="C82" t="inlineStr">
-        <is>
-          <t>GRRR</t>
-        </is>
-      </c>
-      <c r="D82" t="inlineStr">
-        <is>
-          <t>INTA</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>GRVY</t>
+          <t>GSHD</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
+          <t>INTA</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>GTEC</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
           <t>INTU</t>
-        </is>
-      </c>
-      <c r="C83" t="inlineStr">
-        <is>
-          <t>GSHD</t>
-        </is>
-      </c>
-      <c r="D83" t="inlineStr">
-        <is>
-          <t>IVVD</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>GTEC</t>
+          <t>GTIM</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
+          <t>IVVD</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>GTM</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
           <t>JATT</t>
-        </is>
-      </c>
-      <c r="C84" t="inlineStr">
-        <is>
-          <t>GTIM</t>
-        </is>
-      </c>
-      <c r="D84" t="inlineStr">
-        <is>
-          <t>JUNS</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>GTM</t>
+          <t>HALO</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
+          <t>JUNS</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>HCM</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
           <t>KRT</t>
-        </is>
-      </c>
-      <c r="C85" t="inlineStr">
-        <is>
-          <t>HALO</t>
-        </is>
-      </c>
-      <c r="D85" t="inlineStr">
-        <is>
-          <t>LAUR</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>HCM</t>
+          <t>HLNE</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
+          <t>LAUR</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>HNST</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
           <t>LGVN</t>
-        </is>
-      </c>
-      <c r="C86" t="inlineStr">
-        <is>
-          <t>HLNE</t>
-        </is>
-      </c>
-      <c r="D86" t="inlineStr">
-        <is>
-          <t>LOT</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>HNST</t>
+          <t>HPK</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
+          <t>LOT</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>HQWWW</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
           <t>MANH</t>
-        </is>
-      </c>
-      <c r="C87" t="inlineStr">
-        <is>
-          <t>HPK</t>
-        </is>
-      </c>
-      <c r="D87" t="inlineStr">
-        <is>
-          <t>MCAH</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>HQWWW</t>
+          <t>HRZN</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
+          <t>MCAH</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>HTFL</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
           <t>MCRI</t>
-        </is>
-      </c>
-      <c r="C88" t="inlineStr">
-        <is>
-          <t>HRZN</t>
-        </is>
-      </c>
-      <c r="D88" t="inlineStr">
-        <is>
-          <t>MEDP</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>HTFL</t>
+          <t>HUDI</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
+          <t>MEDP</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>HURC</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
           <t>MEOH</t>
-        </is>
-      </c>
-      <c r="C89" t="inlineStr">
-        <is>
-          <t>HUDI</t>
-        </is>
-      </c>
-      <c r="D89" t="inlineStr">
-        <is>
-          <t>MFIN</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>HURC</t>
+          <t>IACO</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
+          <t>MFIN</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>IMC</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
           <t>MKTX</t>
-        </is>
-      </c>
-      <c r="C90" t="inlineStr">
-        <is>
-          <t>IACO</t>
-        </is>
-      </c>
-      <c r="D90" t="inlineStr">
-        <is>
-          <t>MRDN</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>IMC</t>
+          <t>IMCR</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
+          <t>MRDN</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>IMMX</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
           <t>MRVL</t>
-        </is>
-      </c>
-      <c r="C91" t="inlineStr">
-        <is>
-          <t>IMCR</t>
-        </is>
-      </c>
-      <c r="D91" t="inlineStr">
-        <is>
-          <t>MSBIP</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>IMMX</t>
+          <t>IMUX</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
+          <t>MSBIP</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>INBX</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
           <t>NAKA</t>
-        </is>
-      </c>
-      <c r="C92" t="inlineStr">
-        <is>
-          <t>IMUX</t>
-        </is>
-      </c>
-      <c r="D92" t="inlineStr">
-        <is>
-          <t>NBP</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>INBX</t>
+          <t>INDI</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
+          <t>NBP</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>INO</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
           <t>NCI</t>
-        </is>
-      </c>
-      <c r="C93" t="inlineStr">
-        <is>
-          <t>INDI</t>
-        </is>
-      </c>
-      <c r="D93" t="inlineStr">
-        <is>
-          <t>NDAQ</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>INO</t>
+          <t>IPHA</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
+          <t>NDAQ</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>JAN</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
           <t>NMFCZ</t>
-        </is>
-      </c>
-      <c r="C94" t="inlineStr">
-        <is>
-          <t>IPHA</t>
-        </is>
-      </c>
-      <c r="D94" t="inlineStr">
-        <is>
-          <t>NRC</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>JAN</t>
+          <t>JFU</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
+          <t>NRC</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>JKHY</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
           <t>NTNX</t>
-        </is>
-      </c>
-      <c r="C95" t="inlineStr">
-        <is>
-          <t>JFU</t>
-        </is>
-      </c>
-      <c r="D95" t="inlineStr">
-        <is>
-          <t>NTRB</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>JKHY</t>
+          <t>JOYY</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
+          <t>NTRB</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>KELYA</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
           <t>NVAX</t>
-        </is>
-      </c>
-      <c r="C96" t="inlineStr">
-        <is>
-          <t>JOYY</t>
-        </is>
-      </c>
-      <c r="D96" t="inlineStr">
-        <is>
-          <t>NVCT</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>KELYA</t>
+          <t>KLTR</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
+          <t>NVCT</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>KMDA</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
           <t>OCAC</t>
-        </is>
-      </c>
-      <c r="C97" t="inlineStr">
-        <is>
-          <t>KLTR</t>
-        </is>
-      </c>
-      <c r="D97" t="inlineStr">
-        <is>
-          <t>ODTX</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>KMDA</t>
+          <t>KOPN</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
+          <t>ODTX</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>KPRX</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
           <t>OMEX</t>
-        </is>
-      </c>
-      <c r="C98" t="inlineStr">
-        <is>
-          <t>KOPN</t>
-        </is>
-      </c>
-      <c r="D98" t="inlineStr">
-        <is>
-          <t>ONBPO</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>KPRX</t>
+          <t>KRKR</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
+          <t>ONBPO</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>KRNY</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
           <t>ORBS</t>
-        </is>
-      </c>
-      <c r="C99" t="inlineStr">
-        <is>
-          <t>KRKR</t>
-        </is>
-      </c>
-      <c r="D99" t="inlineStr">
-        <is>
-          <t>OTLY</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>KRNY</t>
+          <t>KSPI</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
+          <t>OTLY</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>KWY</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
           <t>OVLY</t>
-        </is>
-      </c>
-      <c r="C100" t="inlineStr">
-        <is>
-          <t>KSPI</t>
-        </is>
-      </c>
-      <c r="D100" t="inlineStr">
-        <is>
-          <t>PAA</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>KWY</t>
+          <t>KZIA</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
+          <t>PAA</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>LECO</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
           <t>PAGP</t>
-        </is>
-      </c>
-      <c r="C101" t="inlineStr">
-        <is>
-          <t>KZIA</t>
-        </is>
-      </c>
-      <c r="D101" t="inlineStr">
-        <is>
-          <t>PANL</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>LECO</t>
+          <t>LEGH</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
+          <t>PANL</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>LEXX</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
           <t>PAYS</t>
-        </is>
-      </c>
-      <c r="C102" t="inlineStr">
-        <is>
-          <t>LEGH</t>
-        </is>
-      </c>
-      <c r="D102" t="inlineStr">
-        <is>
-          <t>PBLS</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>LEXX</t>
+          <t>LIFE</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
+          <t>PBLS</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>LMRI</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
           <t>PEBK</t>
-        </is>
-      </c>
-      <c r="C103" t="inlineStr">
-        <is>
-          <t>LIFE</t>
-        </is>
-      </c>
-      <c r="D103" t="inlineStr">
-        <is>
-          <t>PEP</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>LMRI</t>
+          <t>LPTH</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
+          <t>PEP</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>LSE</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
           <t>PFX</t>
-        </is>
-      </c>
-      <c r="C104" t="inlineStr">
-        <is>
-          <t>LPTH</t>
-        </is>
-      </c>
-      <c r="D104" t="inlineStr">
-        <is>
-          <t>PHOS</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>LSE</t>
+          <t>LTGO</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
+          <t>PHOS</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>LYFT</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
           <t>PLTR</t>
-        </is>
-      </c>
-      <c r="C105" t="inlineStr">
-        <is>
-          <t>LTGO</t>
-        </is>
-      </c>
-      <c r="D105" t="inlineStr">
-        <is>
-          <t>PRGS</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>LYFT</t>
+          <t>MAKO</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
+          <t>PRGS</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>MASS</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
           <t>PRZO</t>
-        </is>
-      </c>
-      <c r="C106" t="inlineStr">
-        <is>
-          <t>MAKO</t>
-        </is>
-      </c>
-      <c r="D106" t="inlineStr">
-        <is>
-          <t>PSEC</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>MASS</t>
+          <t>MBINL</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
+          <t>PSEC</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>MCFT</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
           <t>PSNL</t>
-        </is>
-      </c>
-      <c r="C107" t="inlineStr">
-        <is>
-          <t>MBINL</t>
-        </is>
-      </c>
-      <c r="D107" t="inlineStr">
-        <is>
-          <t>PTLO</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>MCFT</t>
+          <t>MDLZ</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
+          <t>PTLO</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>MELI</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
           <t>PURR</t>
-        </is>
-      </c>
-      <c r="C108" t="inlineStr">
-        <is>
-          <t>MDLZ</t>
-        </is>
-      </c>
-      <c r="D108" t="inlineStr">
-        <is>
-          <t>PXS</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>MELI</t>
+          <t>MGTX</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
+          <t>PXS</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>MGYR</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
           <t>PYPD</t>
-        </is>
-      </c>
-      <c r="C109" t="inlineStr">
-        <is>
-          <t>MGTX</t>
-        </is>
-      </c>
-      <c r="D109" t="inlineStr">
-        <is>
-          <t>RDI</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>MGYR</t>
+          <t>MICC</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
+          <t>RDI</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>MINE</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
           <t>REAX</t>
-        </is>
-      </c>
-      <c r="C110" t="inlineStr">
-        <is>
-          <t>MICC</t>
-        </is>
-      </c>
-      <c r="D110" t="inlineStr">
-        <is>
-          <t>REFI</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>MINE</t>
+          <t>MLAB</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
+          <t>REFI</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>MMED</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
           <t>RENT</t>
-        </is>
-      </c>
-      <c r="C111" t="inlineStr">
-        <is>
-          <t>MLAB</t>
-        </is>
-      </c>
-      <c r="D111" t="inlineStr">
-        <is>
-          <t>RGEN</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>MMED</t>
+          <t>MNKD</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
+          <t>RGEN</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>MNOV</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
           <t>RGLD</t>
-        </is>
-      </c>
-      <c r="C112" t="inlineStr">
-        <is>
-          <t>MNKD</t>
-        </is>
-      </c>
-      <c r="D112" t="inlineStr">
-        <is>
-          <t>RMBI</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>MNOV</t>
+          <t>MOLN</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
+          <t>RMBI</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>MRX</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
           <t>RMNI</t>
-        </is>
-      </c>
-      <c r="C113" t="inlineStr">
-        <is>
-          <t>MOLN</t>
-        </is>
-      </c>
-      <c r="D113" t="inlineStr">
-        <is>
-          <t>RMR</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>MRX</t>
+          <t>MTEX</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
+          <t>RMR</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>MYSE</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
           <t>RNAC</t>
-        </is>
-      </c>
-      <c r="C114" t="inlineStr">
-        <is>
-          <t>MTEX</t>
-        </is>
-      </c>
-      <c r="D114" t="inlineStr">
-        <is>
-          <t>ROIV</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>MYSE</t>
+          <t>MYSZ</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
+          <t>ROIV</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>NAVI</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
           <t>RVMD</t>
-        </is>
-      </c>
-      <c r="C115" t="inlineStr">
-        <is>
-          <t>MYSZ</t>
-        </is>
-      </c>
-      <c r="D115" t="inlineStr">
-        <is>
-          <t>SATA</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>NAVI</t>
+          <t>NEO</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
+          <t>SATA</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>NICM</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
           <t>SBET</t>
-        </is>
-      </c>
-      <c r="C116" t="inlineStr">
-        <is>
-          <t>NEO</t>
-        </is>
-      </c>
-      <c r="D116" t="inlineStr">
-        <is>
-          <t>SBLK</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>NICM</t>
+          <t>NIPG</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
+          <t>SBLK</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>NIQ</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
           <t>SBMT</t>
-        </is>
-      </c>
-      <c r="C117" t="inlineStr">
-        <is>
-          <t>NIPG</t>
-        </is>
-      </c>
-      <c r="D117" t="inlineStr">
-        <is>
-          <t>SEIC</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>NIQ</t>
+          <t>NPAC</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
+          <t>SEIC</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>NSIT</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
           <t>SHIP</t>
-        </is>
-      </c>
-      <c r="C118" t="inlineStr">
-        <is>
-          <t>NPAC</t>
-        </is>
-      </c>
-      <c r="D118" t="inlineStr">
-        <is>
-          <t>SIBN</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>NSIT</t>
+          <t>NTHI</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
+          <t>SIBN</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>NTRA</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
           <t>SIND</t>
-        </is>
-      </c>
-      <c r="C119" t="inlineStr">
-        <is>
-          <t>NTHI</t>
-        </is>
-      </c>
-      <c r="D119" t="inlineStr">
-        <is>
-          <t>SLDE</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>NTRA</t>
+          <t>NWS</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
+          <t>SLDE</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>NWSA</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
           <t>SLS</t>
-        </is>
-      </c>
-      <c r="C120" t="inlineStr">
-        <is>
-          <t>NWS</t>
-        </is>
-      </c>
-      <c r="D120" t="inlineStr">
-        <is>
-          <t>SMJF</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>NWSA</t>
+          <t>NXPL</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
+          <t>SMJF</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>OABI</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
           <t>SMTI</t>
-        </is>
-      </c>
-      <c r="C121" t="inlineStr">
-        <is>
-          <t>NXPL</t>
-        </is>
-      </c>
-      <c r="D121" t="inlineStr">
-        <is>
-          <t>SOFI</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>OABI</t>
+          <t>OBIO</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
+          <t>SOFI</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>OCCI</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
           <t>SRTA</t>
-        </is>
-      </c>
-      <c r="C122" t="inlineStr">
-        <is>
-          <t>OBIO</t>
-        </is>
-      </c>
-      <c r="D122" t="inlineStr">
-        <is>
-          <t>SSMR</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>OCCI</t>
+          <t>OCUL</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
+          <t>SSMR</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>OESX</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
           <t>SSNC</t>
-        </is>
-      </c>
-      <c r="C123" t="inlineStr">
-        <is>
-          <t>OCUL</t>
-        </is>
-      </c>
-      <c r="D123" t="inlineStr">
-        <is>
-          <t>SSRM</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>OESX</t>
+          <t>OGC</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
+          <t>SSRM</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>OGG</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
           <t>STRC</t>
-        </is>
-      </c>
-      <c r="C124" t="inlineStr">
-        <is>
-          <t>OGC</t>
-        </is>
-      </c>
-      <c r="D124" t="inlineStr">
-        <is>
-          <t>STRD</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>OGG</t>
+          <t>OGI</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
+          <t>STRD</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>OMER</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
           <t>STRF</t>
-        </is>
-      </c>
-      <c r="C125" t="inlineStr">
-        <is>
-          <t>OGI</t>
-        </is>
-      </c>
-      <c r="D125" t="inlineStr">
-        <is>
-          <t>STRK</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>OMER</t>
+          <t>OMSE</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
+          <t>STRK</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>OXLCG</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
           <t>SYRE</t>
-        </is>
-      </c>
-      <c r="C126" t="inlineStr">
-        <is>
-          <t>OMSE</t>
-        </is>
-      </c>
-      <c r="D126" t="inlineStr">
-        <is>
-          <t>TAYD</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>OXLCG</t>
+          <t>OXLCM</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
+          <t>TAYD</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>PAYX</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
           <t>TBPH</t>
-        </is>
-      </c>
-      <c r="C127" t="inlineStr">
-        <is>
-          <t>OXLCM</t>
-        </is>
-      </c>
-      <c r="D127" t="inlineStr">
-        <is>
-          <t>TCBX</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>PAYX</t>
+          <t>PBAM</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
+          <t>TCBX</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>PBM</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
           <t>TEM</t>
-        </is>
-      </c>
-      <c r="C128" t="inlineStr">
-        <is>
-          <t>PBAM</t>
-        </is>
-      </c>
-      <c r="D128" t="inlineStr">
-        <is>
-          <t>TII</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>PBM</t>
+          <t>PCTY</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
+          <t>TII</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>PEPG</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
           <t>TOP</t>
-        </is>
-      </c>
-      <c r="C129" t="inlineStr">
-        <is>
-          <t>PCTY</t>
-        </is>
-      </c>
-      <c r="D129" t="inlineStr">
-        <is>
-          <t>TRLV</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>PEPG</t>
+          <t>PHOE</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
+          <t>TRLV</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>PLSE</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
           <t>TRMD</t>
-        </is>
-      </c>
-      <c r="C130" t="inlineStr">
-        <is>
-          <t>PHOE</t>
-        </is>
-      </c>
-      <c r="D130" t="inlineStr">
-        <is>
-          <t>TRON</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>PLSE</t>
+          <t>PLUN</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
+          <t>TRON</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>PMN</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
           <t>TW</t>
-        </is>
-      </c>
-      <c r="C131" t="inlineStr">
-        <is>
-          <t>PLUN</t>
-        </is>
-      </c>
-      <c r="D131" t="inlineStr">
-        <is>
-          <t>TWAV</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>PMN</t>
+          <t>PMTS</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
+          <t>TWAV</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>PMTW</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
           <t>USDE</t>
-        </is>
-      </c>
-      <c r="C132" t="inlineStr">
-        <is>
-          <t>PMTS</t>
-        </is>
-      </c>
-      <c r="D132" t="inlineStr">
-        <is>
-          <t>USDEW</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>PMTW</t>
+          <t>PMVP</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
+          <t>USDEW</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>PPC</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
           <t>VGNT</t>
-        </is>
-      </c>
-      <c r="C133" t="inlineStr">
-        <is>
-          <t>PMVP</t>
-        </is>
-      </c>
-      <c r="D133" t="inlineStr">
-        <is>
-          <t>VMET</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>PPC</t>
+          <t>PRAA</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
+          <t>VMET</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>PRCH</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
           <t>VOGX</t>
-        </is>
-      </c>
-      <c r="C134" t="inlineStr">
-        <is>
-          <t>PRAA</t>
-        </is>
-      </c>
-      <c r="D134" t="inlineStr">
-        <is>
-          <t>VOXR</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>PRCH</t>
+          <t>PRHI</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
+          <t>VOXR</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>PRLD</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
           <t>WHK</t>
-        </is>
-      </c>
-      <c r="C135" t="inlineStr">
-        <is>
-          <t>PRHI</t>
-        </is>
-      </c>
-      <c r="D135" t="inlineStr">
-        <is>
-          <t>XXI</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>PRLD</t>
+          <t>PROV</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>PROV</t>
+          <t>XXI</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
@@ -3719,183 +3719,183 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>TEAM</t>
+          <t>AEHL</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>FCUV</t>
+          <t>ORMP</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>DAAQU</t>
+          <t>IXHL</t>
         </is>
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>ABOS</t>
+          <t>KGEI</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
+          <t>RDZN</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>TEAM</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
           <t>CABA</t>
         </is>
       </c>
-      <c r="B152" t="inlineStr">
-        <is>
-          <t>INCY</t>
-        </is>
-      </c>
-      <c r="C152" t="inlineStr">
-        <is>
-          <t>IXHL</t>
-        </is>
-      </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>ANIX</t>
+          <t>ACRV</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>IOVA</t>
+          <t>DAAQU</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>APA</t>
+          <t>RCMT</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>KGEI</t>
+          <t>LNSR</t>
         </is>
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t>GCL</t>
+          <t>YDES</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>CGEM</t>
+          <t>IPST</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>BFRI</t>
+          <t>ABOS</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>GWRS</t>
+          <t>ISNRW</t>
         </is>
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>RIGL</t>
+          <t>IOVA</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>ACHV</t>
+          <t>BRR</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>CHRD</t>
+          <t>AVAH</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>CPRT</t>
+          <t>MF</t>
         </is>
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t>HTHT</t>
+          <t>INCY</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>ISNRW</t>
+          <t>NBTX</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>YDES</t>
+          <t>CLYM</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>ACRV</t>
+          <t>NERV</t>
         </is>
       </c>
       <c r="D156" t="inlineStr">
         <is>
-          <t>IPST</t>
+          <t>NCT</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>CSTE</t>
+          <t>CGEM</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>LNSR</t>
+          <t>ALEC</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>BIXIW</t>
+          <t>GNLN</t>
         </is>
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>NBTX</t>
+          <t>RIGL</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>BRR</t>
+          <t>GWRS</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>MORN</t>
+          <t>CSTE</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>RDZN</t>
+          <t>CHRN</t>
         </is>
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>CHRN</t>
+          <t>HTHT</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>ORMP</t>
+          <t>MORN</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
@@ -3905,68 +3905,68 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>AVAH</t>
+          <t>CHRD</t>
         </is>
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>HWH</t>
+          <t>CPRT</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>NCT</t>
+          <t>FCUV</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>ALEC</t>
+          <t>GCL</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>GNLN</t>
+          <t>BIXIW</t>
         </is>
       </c>
       <c r="D160" t="inlineStr">
         <is>
-          <t>RCMT</t>
+          <t>KBSX</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>AEHL</t>
+          <t>FORTY</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>MF</t>
+          <t>BFRI</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>FORTY</t>
+          <t>ANIX</t>
         </is>
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>KBSX</t>
+          <t>ACHV</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>NERV</t>
+          <t>APA</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>CLYM</t>
+          <t>HWH</t>
         </is>
       </c>
       <c r="C162" t="inlineStr"/>

</xml_diff>

<commit_message>
Momentum scan results 2026-08-26
</commit_message>
<xml_diff>
--- a/results/momentum_merged_latest.xlsx
+++ b/results/momentum_merged_latest.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D161"/>
+  <dimension ref="A1:D183"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -441,12 +441,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>AACI</t>
+          <t>ACAD</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>ABOS</t>
+          <t>ABCL</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -456,80 +456,80 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>AIOS</t>
+          <t>AEC</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>ACRS</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
           <t>ABNB</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>ACAD</t>
-        </is>
-      </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>AMOD</t>
+          <t>AD</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>AIXC</t>
+          <t>AIDX</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>ABXL</t>
+          <t>ACU</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>ACET</t>
+          <t>ABSI</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>ANAB</t>
+          <t>BEAM</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>ALCO</t>
+          <t>ATLX</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>ACT</t>
+          <t>AKTS</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>ACFN</t>
+          <t>ACCL</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>BHFAL</t>
+          <t>BRNS</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>ATLX</t>
+          <t>ATOS</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ADP</t>
+          <t>ALLO</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -539,63 +539,63 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>CENN</t>
+          <t>BTBT</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>ATOS</t>
+          <t>AWRE</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>AKTS</t>
+          <t>ALOT</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>ADAG</t>
+          <t>ACIU</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>DXLG</t>
+          <t>FLD</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>BTOC</t>
+          <t>BGIN</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>ALVO</t>
+          <t>APPN</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>ADAMH</t>
+          <t>ADAMI</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>EEIQ</t>
+          <t>GLSI</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>DETX</t>
+          <t>BREZ</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>AMAN</t>
+          <t>ARCT</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -605,19 +605,19 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>ELVR</t>
+          <t>IBRX</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>DUKR</t>
+          <t>BWIV</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>AMCR</t>
+          <t>AREC</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -627,85 +627,85 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>FCFS</t>
+          <t>IONS</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>ELPW</t>
+          <t>CRGO</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>AMGN</t>
+          <t>ASBP</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>ADBE</t>
+          <t>ADPT</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>GMTL</t>
+          <t>KTTA</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>FABC</t>
+          <t>DUO</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>ANL</t>
+          <t>ASMB</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>ADSK</t>
+          <t>ADUS</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>HNRG</t>
+          <t>KXIN</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>FINW</t>
+          <t>EEIQ</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>APA</t>
+          <t>ASST</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>ADUS</t>
+          <t>AEI</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>KXIN</t>
+          <t>LBTYK</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>GLE</t>
+          <t>ELPW</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>APPF</t>
+          <t>ASUR</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -715,232 +715,232 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>LNZA</t>
+          <t>LEE</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>GLSI</t>
+          <t>FULC</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>APPN</t>
+          <t>AVO</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>AGYS</t>
+          <t>AFRM</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>METC</t>
+          <t>LNZA</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>GMRS</t>
+          <t>GMTL</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>ARCT</t>
+          <t>AXIN</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>ALGS</t>
+          <t>AGEN</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>PPIH</t>
+          <t>LUCD</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>GYRE</t>
+          <t>GRDX</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>ASMB</t>
+          <t>AYA</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>ALLR</t>
+          <t>AGMH</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>PUSA</t>
+          <t>NGEN</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>HROW</t>
+          <t>GRSD</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>ASST</t>
+          <t>BBW</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>ALMR</t>
+          <t>AGPU</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>RAND</t>
+          <t>NTLA</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>IONS</t>
+          <t>HAO</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>ATLCL</t>
+          <t>BCDA</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>ALPX</t>
+          <t>AGYS</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>SCNI</t>
+          <t>NYXH</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>KIDZ</t>
+          <t>HNRG</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>AVAH</t>
+          <t>BDSX</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>ALRM</t>
+          <t>AIFC</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>TIL</t>
+          <t>OCGN</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>LASE</t>
+          <t>HROW</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>AVO</t>
+          <t>BEEP</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>AMCX</t>
+          <t>ALGS</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>VIR</t>
+          <t>OCS</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>LKFT</t>
+          <t>INAB</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>AWR</t>
+          <t>BHAV</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>AMLX</t>
+          <t>ALM</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>LUCD</t>
+          <t>PPBT</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>BAFN</t>
+          <t>INVE</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>AMPH</t>
+          <t>BID</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>ALZN</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>BCDA</t>
+          <t>PSNYW</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>ANGX</t>
+          <t>IPVV</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>OCS</t>
+          <t>BKNG</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>BKNG</t>
+          <t>AMCR</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>ANIK</t>
+          <t>PTN</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>OFRM</t>
+          <t>KIDZ</t>
         </is>
       </c>
     </row>
@@ -952,3011 +952,3487 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>AQST</t>
+          <t>AMCX</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>PLBY</t>
+          <t>RAND</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>BMEA</t>
+          <t>KLRS</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>ARCC</t>
+          <t>BMEA</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>PPBT</t>
+          <t>AMLX</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>BMNP</t>
+          <t>REED</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>ARLP</t>
+          <t>LASE</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>RVSN</t>
+          <t>BMNR</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>BMNR</t>
+          <t>AMPH</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>ARTNA</t>
+          <t>RXRX</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>SJ</t>
+          <t>LBTYA</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>BOW</t>
+          <t>BRNX</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>ARX</t>
+          <t>AMPL</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>TPST</t>
+          <t>SCNI</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>BR</t>
+          <t>METC</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>ASND</t>
+          <t>BULL</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>VYGR</t>
+          <t>AMR</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>BRCB</t>
+          <t>TCBIO</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>ATLO</t>
+          <t>PSIG</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>WHK</t>
+          <t>BWBBP</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>BRZE</t>
+          <t>ANDG</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>ATRC</t>
+          <t>TRDA</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>WSE</t>
+          <t>RENX</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>BSVN</t>
+          <t>BWIN</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>AUGO</t>
+          <t>ANGO</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>BTBD</t>
+          <t>USAR</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>AUPH</t>
+          <t>SBAC</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>BTCS</t>
+          <t>CAAS</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>AURA</t>
+          <t>ANGX</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>BTCT</t>
+          <t>SGML</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>AUTL</t>
+          <t>CAI</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>CAAS</t>
+          <t>APA</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>AVBC</t>
+          <t>SPCX</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>CAKE</t>
+          <t>CAN</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>AVIR</t>
+          <t>APAC</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>CCEC</t>
+          <t>TPST</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>AVR</t>
+          <t>CBAT</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>CCU</t>
+          <t>APGE</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>BANL</t>
+          <t>CCCC</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
+          <t>APLM</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>CCG</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>AQST</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
           <t>CDLR</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>BATRA</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>CEG</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>BBNX</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>CELH</t>
+          <t>AR</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>BCIC</t>
+          <t>CDNA</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>CGAU</t>
+          <t>ARCC</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>BEBE</t>
+          <t>CDZI</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>CHDN</t>
+          <t>ARLP</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>BEEP</t>
+          <t>CELU</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>CHTRP</t>
+          <t>ARVN</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>BIIB</t>
+          <t>CENT</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>CING</t>
+          <t>ARWR</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>BL</t>
+          <t>CFFI</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>CLAR</t>
+          <t>ARX</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>BLKB</t>
+          <t>CGEN</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>CLIR</t>
+          <t>ATKR</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>BLSH</t>
+          <t>CHCI</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>CMMB</t>
+          <t>ATLO</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>BMRN</t>
+          <t>CHRN</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>CMPS</t>
+          <t>ATR</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>BNGO</t>
+          <t>CHSCO</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>COIN</t>
+          <t>ATRA</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>BNTC</t>
+          <t>CHTRP</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>CORT</t>
+          <t>AU</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>BPRN</t>
+          <t>CING</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>COUR</t>
+          <t>AUGO</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>BRNX</t>
+          <t>CLPT</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>COYA</t>
+          <t>AUPH</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>BSY</t>
+          <t>CMCSA</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>CPB</t>
+          <t>AUTL</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>BTU</t>
+          <t>CMMB</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>CRBP</t>
+          <t>BATRA</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>BWBBP</t>
+          <t>CNTB</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>CRON</t>
+          <t>BATRK</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>BWIN</t>
+          <t>CNTY</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>CSHR</t>
+          <t>BBOT</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>CABA</t>
+          <t>COKE</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>CSWC</t>
+          <t>BCIC</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>CARG</t>
+          <t>CORT</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>CTAS</t>
+          <t>BCYC</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>CARL</t>
+          <t>COUR</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>CTW</t>
+          <t>BDTX</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>CART</t>
+          <t>COYA</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>CVSA</t>
+          <t>BEEM</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>CBFV</t>
+          <t>CPBI</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>CYPH</t>
+          <t>BFRI</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>CCC</t>
+          <t>CPIX</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>CZNC</t>
+          <t>BGDE</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>CCCC</t>
+          <t>CRBP</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>DEFT</t>
+          <t>BIIB</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>CCG</t>
+          <t>CRON</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>DFDV</t>
+          <t>BLSH</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>CCLD</t>
+          <t>CRSP</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>DHCNI</t>
+          <t>BMNP</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>CCNEP</t>
+          <t>CSTE</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>DLTR</t>
+          <t>BNGO</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>CERT</t>
+          <t>CSTL</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>DMC</t>
+          <t>BOXL</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>CGBD</t>
+          <t>CTOR</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>DSGX</t>
+          <t>BPYPP</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>CGEM</t>
+          <t>CURX</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>DTCX</t>
+          <t>BRLS</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>CGEN</t>
+          <t>CUVL</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>DWTX</t>
+          <t>BSBR</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>CHRD</t>
+          <t>CVSA</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>EDRY</t>
+          <t>BTBD</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>CHRN</t>
+          <t>CYCN</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>ELVN</t>
+          <t>BTCS</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>CIGI</t>
+          <t>DFDV</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>ENGS</t>
+          <t>BTCT</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>CIMP</t>
+          <t>DFDVW</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>EOLS</t>
+          <t>BTGO</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>CMCSA</t>
+          <t>DMAA</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>EPRX</t>
+          <t>CABA</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>CME</t>
+          <t>DNLI</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>ERIE</t>
+          <t>CADL</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>CNET</t>
+          <t>DSGN</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>EXE</t>
+          <t>CAII</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>CNOBP</t>
+          <t>DTI</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>EXPE</t>
+          <t>CARL</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>CNR</t>
+          <t>DWTX</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>EXPO</t>
+          <t>CCSI</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>CNXC</t>
+          <t>ECBK</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>FDMT</t>
+          <t>CDIO</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>COKE</t>
+          <t>EDIT</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>FDSB</t>
+          <t>CEG</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>CPIX</t>
+          <t>EDRY</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>FHTX</t>
+          <t>CELH</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>CRMD</t>
+          <t>ELUT</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>FIVE</t>
+          <t>CENN</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>CRVL</t>
+          <t>EML</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>FIZZ</t>
+          <t>CGAU</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>CTSH</t>
+          <t>ENGS</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>FLNT</t>
+          <t>CGEM</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>CUB</t>
+          <t>ENTX</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>FRPT</t>
+          <t>CHDN</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>CURX</t>
+          <t>EOLS</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>FSUN</t>
+          <t>CHRD</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>DAAQ</t>
+          <t>EPRX</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>FSV</t>
+          <t>CHYM</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>DASH</t>
+          <t>EVER</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>FTH</t>
+          <t>CIMP</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>DBX</t>
+          <t>FEAM</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>FVN</t>
+          <t>CLBK</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>DDI</t>
+          <t>FLXS</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>FWDI</t>
+          <t>CLLS</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>DERM</t>
+          <t>FORR</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>FWONA</t>
+          <t>CLPS</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>DMLP</t>
+          <t>FORTY</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>FWONK</t>
+          <t>CLYM</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>DNUT</t>
+          <t>FRHC</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>GBDC</t>
+          <t>CMPS</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>DOCU</t>
+          <t>FSEA</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>GCBC</t>
+          <t>CNOBP</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>DOX</t>
+          <t>FUTU</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>GECC</t>
+          <t>CNR</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>DRMA</t>
+          <t>FWDI</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>GENB</t>
+          <t>CNXC</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>DSC</t>
+          <t>GEN</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>GILD</t>
+          <t>COIN</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>ECBK</t>
+          <t>GENB</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>GLAD</t>
+          <t>COR</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>ECCU</t>
+          <t>GOLD</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>GSHD</t>
+          <t>CRAI</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>ECPG</t>
+          <t>GRFS</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>GWRS</t>
+          <t>CRMD</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>EHLD</t>
+          <t>HAVA</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>HAIN</t>
+          <t>CRNX</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>ELBM</t>
+          <t>HELP</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>HAS</t>
+          <t>CTRM</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>ELE</t>
+          <t>HITI</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>HBANL</t>
+          <t>CTSH</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>EMBJ</t>
+          <t>HNNA</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>HELP</t>
+          <t>CTW</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>EML</t>
+          <t>HNST</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>HNST</t>
+          <t>CWBC</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>ENTX</t>
+          <t>HOOD</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>HNVR</t>
+          <t>CXII</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>EROK</t>
+          <t>HSLV</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>HSDT</t>
+          <t>DAAQ</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>ETON</t>
+          <t>HWCPZ</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>HTO</t>
+          <t>DASH</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>EVAX</t>
+          <t>HYPD</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>HURN</t>
+          <t>DERM</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>EWTX</t>
+          <t>IBKR</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
+          <t>DJCO</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
           <t>IDYA</t>
-        </is>
-      </c>
-      <c r="D71" t="inlineStr">
-        <is>
-          <t>EXFY</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>IKT</t>
+          <t>DOX</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>EXLS</t>
+          <t>IFRX</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
+          <t>DRMA</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
           <t>ILMN</t>
-        </is>
-      </c>
-      <c r="D72" t="inlineStr">
-        <is>
-          <t>FAST</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>IMPP</t>
+          <t>DXCM</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>FBRX</t>
+          <t>IMC</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>INBX</t>
+          <t>DYN</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>FCBC</t>
+          <t>IMMX</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>INMB</t>
+          <t>EBON</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>FCUV</t>
+          <t>IMNM</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>IOSP</t>
+          <t>EFOR</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>FENC</t>
+          <t>INBX</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
+          <t>EIKN</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>INTS</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>ELE</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
           <t>IRD</t>
-        </is>
-      </c>
-      <c r="B75" t="inlineStr">
-        <is>
-          <t>FERA</t>
-        </is>
-      </c>
-      <c r="C75" t="inlineStr">
-        <is>
-          <t>IVA</t>
-        </is>
-      </c>
-      <c r="D75" t="inlineStr">
-        <is>
-          <t>FIVN</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>JANX</t>
+          <t>ETON</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>FNKO</t>
+          <t>ITIC</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>JKHY</t>
+          <t>EXOZ</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>FORR</t>
+          <t>IXHL</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>JRSH</t>
+          <t>FBLA</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>FOSL</t>
+          <t>JANX</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>KBSX</t>
+          <t>FBRX</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>FOX</t>
+          <t>JAZZ</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>KIDS</t>
+          <t>FCUV</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>FOXA</t>
+          <t>JKHY</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>KROS</t>
+          <t>FENC</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>FRSH</t>
+          <t>KOYN</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
+          <t>FGI</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>KSPI</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>FIGR</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
           <t>KURA</t>
-        </is>
-      </c>
-      <c r="B79" t="inlineStr">
-        <is>
-          <t>FSSL</t>
-        </is>
-      </c>
-      <c r="C79" t="inlineStr">
-        <is>
-          <t>KYNB</t>
-        </is>
-      </c>
-      <c r="D79" t="inlineStr">
-        <is>
-          <t>FTDR</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>LCUT</t>
+          <t>FIZZ</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>FXAC</t>
+          <t>KYMR</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>LECO</t>
+          <t>FLGT</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>GAINI</t>
+          <t>KYNB</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>LEGH</t>
+          <t>FOX</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>GCL</t>
+          <t>LECO</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>LIEN</t>
+          <t>FOXA</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>GCT</t>
+          <t>LIFE</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>LIFE</t>
+          <t>FRD</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>GLBS</t>
+          <t>LKFT</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>LLYVA</t>
+          <t>FRNM</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>GLIBA</t>
+          <t>LOT</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>LLYVK</t>
+          <t>FSSL</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>GLIBK</t>
+          <t>LUNG</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>LOT</t>
+          <t>FTDR</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>GLMD</t>
+          <t>MAKO</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>MAKO</t>
+          <t>FXAC</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>GLNG</t>
+          <t>MBINL</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>MASS</t>
+          <t>GAINI</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>GO</t>
+          <t>MCGA</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>MDLZ</t>
+          <t>GALT</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>GOODO</t>
+          <t>MCRI</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>METCZ</t>
+          <t>GCBC</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>GRAL</t>
+          <t>MEDP</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>MGTX</t>
+          <t>GCT</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>GROW</t>
+          <t>METCI</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
+          <t>GECC</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
           <t>MICC</t>
-        </is>
-      </c>
-      <c r="D86" t="inlineStr">
-        <is>
-          <t>GRVY</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>MINE</t>
+          <t>GILD</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>HALO</t>
+          <t>MKLY</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>MNOV</t>
+          <t>GLAD</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>HHS</t>
+          <t>MKLYU</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>MSTR</t>
+          <t>GLE</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>HOWL</t>
+          <t>MNOV</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>MTCH</t>
+          <t>GLIBA</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>HQI</t>
+          <t>MRKR</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>NAKA</t>
+          <t>GLIBK</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>HRMY</t>
+          <t>MRNA</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>NCI</t>
+          <t>GLNG</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>HSIC</t>
+          <t>MRVI</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>NCNO</t>
+          <t>GMAB</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>HTFL</t>
+          <t>MSTR</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>NDAQ</t>
+          <t>GO</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>HXHX</t>
+          <t>MTCH</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>NESR</t>
+          <t>GRAL</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>HYPD</t>
+          <t>MWYN</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>NEWTH</t>
+          <t>GRVY</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>ICFI</t>
+          <t>MYSE</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>NGNE</t>
+          <t>GWRS</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>ICUI</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>NKTR</t>
+          <t>HAIN</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>IMXI</t>
+          <t>NFLX</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>NTNX</t>
+          <t>HALO</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>INBKZ</t>
+          <t>NGNE</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>NTRB</t>
+          <t>HAS</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>INCY</t>
+          <t>NIPG</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>NVCT</t>
+          <t>HBIO</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>INO</t>
+          <t>NMFCZ</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>NWS</t>
+          <t>HFFG</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>INTU</t>
+          <t>NRIX</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>OCCIN</t>
+          <t>HHS</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>IOND</t>
+          <t>NSLRL</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>OGG</t>
+          <t>HLNE</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>IRON</t>
+          <t>NTRA</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>ORBS</t>
+          <t>HOWL</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>ITIC</t>
+          <t>NUTX</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>OTLY</t>
+          <t>HPK</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>JAN</t>
+          <t>NVAX</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>OVBC</t>
+          <t>HQ</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>JATT</t>
+          <t>NVCT</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>PANL</t>
+          <t>HQWWW</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>JCAP</t>
+          <t>NXPL</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>PAX</t>
+          <t>HQY</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>JG</t>
+          <t>OESX</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>PAYS</t>
+          <t>HRMY</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>JJSF</t>
+          <t>OGG</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>PAYX</t>
+          <t>HSCS</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>JSM</t>
+          <t>OMEX</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>PBAM</t>
+          <t>HSIC</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>KDP</t>
+          <t>ONBPO</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>PEGA</t>
+          <t>HTHT</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>KMDA</t>
+          <t>ONBPP</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>PEP</t>
+          <t>HUIZ</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>KNSA</t>
+          <t>ORMP</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>PFX</t>
+          <t>IBEX</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>KPRX</t>
+          <t>OTAI</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>PHOS</t>
+          <t>IDAI</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>KRKR</t>
+          <t>OWLS</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>PNRG</t>
+          <t>IDCC</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>KRNY</t>
+          <t>OXLCZ</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>PROV</t>
+          <t>III</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>KRT</t>
+          <t>PAYS</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>PRQR</t>
+          <t>IMCR</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>KSPI</t>
+          <t>PBYI</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>PS</t>
+          <t>IMMR</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>KWY</t>
+          <t>PECE</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>PTGX</t>
+          <t>INCY</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>LARK</t>
+          <t>PEPG</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>PURR</t>
+          <t>INMB</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>LBRX</t>
+          <t>PGEN</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>PXS</t>
+          <t>INO</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>LFVN</t>
+          <t>PHIO</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>QTTB</t>
+          <t>INTA</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>LMNR</t>
+          <t>PMN</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>RACD</t>
+          <t>IOND</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>LNSR</t>
+          <t>PMTW</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>RAPP</t>
+          <t>IOVA</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>LYFT</t>
+          <t>PRE</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>RBKB</t>
+          <t>IPHA</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>MAZE</t>
+          <t>PRME</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>RGEN</t>
+          <t>IRON</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>MBBC</t>
+          <t>PRTA</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>RGLD</t>
+          <t>IRTC</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>MELI</t>
+          <t>PRZO</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>RMBI</t>
+          <t>JAB</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>MESH</t>
+          <t>PS</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>RUM</t>
+          <t>JAN</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>MGNI</t>
+          <t>PSEC</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>SABR</t>
+          <t>JATT</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>MKTX</t>
+          <t>PTC</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>SATA</t>
+          <t>JCAP</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>MNDY</t>
+          <t>PURR</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>SBC</t>
+          <t>JCTC</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>MNKD</t>
+          <t>PXLW</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>SBET</t>
+          <t>JG</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>MODD</t>
+          <t>PYPL</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>SBLK</t>
+          <t>JSM</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>MORN</t>
+          <t>QURE</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>SBMT</t>
+          <t>KMDA</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>MRDN</t>
+          <t>RACD</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>SCTX</t>
+          <t>KNSA</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>MSEX</t>
+          <t>RAPP</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>SCYX</t>
+          <t>KRKR</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>RCBC</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>SEIC</t>
+          <t>KRNY</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>MTEX</t>
+          <t>RCKT</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>SHIP</t>
+          <t>KROS</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>MYSZ</t>
+          <t>RDI</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>SLDE</t>
+          <t>KRRO</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>NAVI</t>
+          <t>RGEN</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>SLNHP</t>
+          <t>KRT</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>NAVN</t>
+          <t>RIGL</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>SPRB</t>
+          <t>KYTX</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>NCT</t>
+          <t>RILYG</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>SPT</t>
+          <t>KZIA</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>NHP</t>
+          <t>RMCO</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>SRRK</t>
+          <t>LARK</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>NIQ</t>
+          <t>RNXT</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>SRTS</t>
+          <t>LBRX</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>NMFC</t>
+          <t>RUM</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>SSMR</t>
+          <t>LEGH</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>NMIH</t>
+          <t>SANA</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>STRC</t>
+          <t>LEXX</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>NPT</t>
+          <t>SATA</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>STRD</t>
+          <t>LIEN</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>NRDS</t>
+          <t>SBET</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>STRF</t>
+          <t>LILAK</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>NTHI</t>
+          <t>SBLK</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>STRK</t>
+          <t>LIME</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>NTWOW</t>
+          <t>SCTX</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>STTK</t>
+          <t>LKQ</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>NWGL</t>
+          <t>SEGG</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>SY</t>
+          <t>LLYVA</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>NWSA</t>
+          <t>SEIC</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>TIPT</t>
+          <t>LLYVK</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>OABI</t>
+          <t>SIND</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>TOP</t>
+          <t>LTGO</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>OBIO</t>
+          <t>SLDB</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>TRGS</t>
+          <t>LXEO</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>OCSL</t>
+          <t>SMTI</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>TRIN</t>
+          <t>MANH</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>OCUL</t>
+          <t>SPRB</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>TRLV</t>
+          <t>MASS</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>OESX</t>
+          <t>SPT</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>TRNI</t>
+          <t>MAZE</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>OGC</t>
+          <t>SRRK</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>TRON</t>
+          <t>MCFT</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>OGI</t>
+          <t>SSRM</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>TWAV</t>
+          <t>MDIA</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>OMDA</t>
+          <t>STDN</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>VMET</t>
+          <t>MDXG</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>OMER</t>
+          <t>STRA</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>VOGX</t>
+          <t>MDXH</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>OPRT</t>
+          <t>STRD</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>VOXR</t>
+          <t>MELI</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>ORMP</t>
+          <t>SWVL</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>XRPN</t>
+          <t>MESO</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>OTAI</t>
+          <t>SYRE</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>XXI</t>
+          <t>METCZ</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>OVID</t>
+          <t>TBLD</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>YORW</t>
+          <t>MF</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>OXLC</t>
+          <t>TCPC</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>OXLCI</t>
+          <t>MFIN</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>PAA</t>
+          <t>TIGR</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>PAGP</t>
+          <t>MGNI</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>PBLS</t>
+          <t>TNXP</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>PBYI</t>
+          <t>MGTX</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>PDEX</t>
+          <t>TRLV</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>PEBK</t>
+          <t>MKTX</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>PEPG</t>
+          <t>VERU</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>PGEN</t>
+          <t>MLAB</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>PHVS</t>
+          <t>VIR</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>PMTS</t>
+          <t>MMSI</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>PMTW</t>
+          <t>VMET</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>PMVP</t>
+          <t>MMTX</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>PPTA</t>
+          <t>VOR</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>PRAA</t>
+          <t>MNKD</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>PRLD</t>
+          <t>XNCR</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>PRPO</t>
+          <t>MNSB</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>PSUS</t>
+          <t>MODD</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>PTLO</t>
+          <t>MRVL</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>PTORU</t>
+          <t>MSFT</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>PYPD</t>
+          <t>MSGY</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>RCBC</t>
+          <t>NAVI</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>RCEL</t>
+          <t>NCO</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>RCKT</t>
+          <t>NCT</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>RCMT</t>
+          <t>NEOV</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>RDZN</t>
+          <t>NERV</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>REFI</t>
+          <t>NESR</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>RILYG</t>
+          <t>NEWTG</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>RMCO</t>
+          <t>NEXM</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>RNA</t>
+          <t>NHPBP</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>ROKU</t>
+          <t>NIQ</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>ROP</t>
+          <t>NKTR</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>RPD</t>
+          <t>NKTX</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>RPRX</t>
+          <t>NSPR</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>RRGB</t>
+          <t>NSTS</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>RWAY</t>
+          <t>NTHI</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>SAFT</t>
+          <t>NVA</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>SAV</t>
+          <t>NVCR</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>SBGI</t>
+          <t>NWGL</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>SENEA</t>
+          <t>NWS</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>SFBC</t>
+          <t>NWSA</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>SGHT</t>
+          <t>OGC</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>SHOP</t>
+          <t>OGI</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>SIEB</t>
+          <t>OMSE</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>SIND</t>
+          <t>ONC</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>SLN</t>
+          <t>OPRX</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>SLNG</t>
+          <t>ORBS</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>SMSI</t>
+          <t>OVBC</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>SOGP</t>
+          <t>OVID</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>SOHU</t>
+          <t>OXLC</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>SPSC</t>
+          <t>OXLCG</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>SSNC</t>
+          <t>OXLCN</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>SSP</t>
+          <t>OZKAP</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>SSRM</t>
+          <t>PANL</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>STLN</t>
+          <t>PAX</t>
         </is>
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>STOK</t>
+          <t>PCTY</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>STRA</t>
+          <t>PCYO</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>SUNC</t>
+          <t>PGY</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>SVAQ</t>
+          <t>PLRX</t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>SVRN</t>
+          <t>PLSE</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>TARS</t>
+          <t>PMTS</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>TCBX</t>
+          <t>PPC</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>TEAM</t>
+          <t>PPTA</t>
         </is>
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>TECH</t>
+          <t>PRCH</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>TII</t>
+          <t>PRDO</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>TILE</t>
+          <t>PRHI</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>TLF</t>
+          <t>PROV</t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>TLSA</t>
+          <t>PRTS</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>TNON</t>
+          <t>PUBM</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>TNXP</t>
+          <t>QMCO</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>TP</t>
+          <t>QNBC</t>
         </is>
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>TPG</t>
+          <t>RANI</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>TRI</t>
+          <t>RCEL</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>TRMB</t>
+          <t>RCMT</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>TW</t>
+          <t>RDNT</t>
         </is>
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>VCTR</t>
+          <t>RDVT</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>VSNT</t>
+          <t>REA</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>WTW</t>
+          <t>RECT</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>XNCR</t>
+          <t>REFI</t>
         </is>
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>XRN</t>
+          <t>REPL</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>YDES</t>
+          <t>RFAIU</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>YSWY</t>
+          <t>RGLD</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>ODTX</t>
+          <t>RILYN</t>
         </is>
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t>HTHT</t>
+          <t>RLYB</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>SLS</t>
+          <t>RMNI</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>BFRI</t>
+          <t>RNA</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>BYND</t>
+          <t>RNAC</t>
         </is>
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>AEHL</t>
+          <t>ROIV</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>LTGO</t>
+          <t>ROKU</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>LGVN</t>
+          <t>RPRX</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>FBLG</t>
+          <t>RWAYI</t>
         </is>
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>HQ</t>
+          <t>RWAYL</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>MF</t>
+          <t>SAV</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>FRNM</t>
+          <t>SBC</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>DFDVW</t>
+          <t>SBGI</t>
         </is>
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>ISNRW</t>
+          <t>SCZM</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>DAAQU</t>
+          <t>SDGR</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>ATRA</t>
+          <t>SEV</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>ACB</t>
+          <t>SFBC</t>
         </is>
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>AIFC</t>
+          <t>SGMT</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>CITR</t>
+          <t>SGP</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>SMJF</t>
+          <t>SHIP</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>PRHI</t>
+          <t>SHOP</t>
         </is>
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t>IXHL</t>
+          <t>SJ</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>SELF</t>
+          <t>SLMBP</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>ACIU</t>
+          <t>SLN</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>ALM</t>
+          <t>SLNG</t>
         </is>
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>RDI</t>
+          <t>SMCI</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>PLSE</t>
+          <t>SMCIP</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>NERV</t>
+          <t>SNY</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>BRR</t>
+          <t>SOCA</t>
         </is>
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t>IMC</t>
+          <t>SOFI</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>MFI</t>
+          <t>SOTK</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>CELU</t>
+          <t>SPTX</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>PPC</t>
+          <t>SRPT</t>
         </is>
       </c>
       <c r="D156" t="inlineStr">
         <is>
-          <t>IVVD</t>
+          <t>STOK</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>RNAC</t>
+          <t>STRK</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>ALEC</t>
+          <t>STRZ</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>USDE</t>
+          <t>STTK</t>
         </is>
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>HBIO</t>
+          <t>SVRN</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>LSE</t>
+          <t>SWIM</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>EXOZ</t>
+          <t>SWKHL</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>AIFA</t>
+          <t>SY</t>
         </is>
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>HQWWW</t>
+          <t>TAOX</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>GTEC</t>
+          <t>TAYD</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>ACRV</t>
+          <t>TEAM</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>HITI</t>
+          <t>TECX</t>
         </is>
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>FLXS</t>
+          <t>TII</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>BRLS</t>
+          <t>TILE</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>IMMX</t>
+          <t>TKNO</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>DUOL</t>
+          <t>TLRY</t>
         </is>
       </c>
       <c r="D160" t="inlineStr">
         <is>
-          <t>INTS</t>
+          <t>TLX</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>AMR</t>
+          <t>TMC</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
         <is>
+          <t>TORO</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>TPG</t>
+        </is>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>TRIN</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>TRMD</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>TRON</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>USDE</t>
+        </is>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>VOGX</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>VSNT</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>VYGR</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>XIIIU</t>
+        </is>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>XRN</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>XRPN</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>XXI</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>ZSTK</t>
+        </is>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>KBSX</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>BIVI</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>NTWOW</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>MFP</t>
+        </is>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>VOXR</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>GCL</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>OMER</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>PSNL</t>
+        </is>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>ODTX</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>RFAI</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>BRR</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>GSHD</t>
+        </is>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>BAFN</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>RDACU</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>ACB</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>BNTX</t>
+        </is>
+      </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>HSDT</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>BNC</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>CSHR</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>HOLO</t>
+        </is>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>EXFY</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>OPK</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>PRPO</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>IVVD</t>
+        </is>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>EZRA</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>ASPCU</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>NTRB</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>AEHL</t>
+        </is>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>CYPH</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>QTTB</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>LNSR</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>ATRC</t>
+        </is>
+      </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>TEM</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>NAKA</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>DTCX</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>USAU</t>
+        </is>
+      </c>
+      <c r="D173" t="inlineStr">
+        <is>
+          <t>ALEC</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>PRLD</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>DEFT</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>DAAQU</t>
+        </is>
+      </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>APPF</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>SELF</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>BTU</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>MFI</t>
+        </is>
+      </c>
+      <c r="D175" t="inlineStr">
+        <is>
+          <t>BANL</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>AVAH</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>HTFL</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>SBMT</t>
+        </is>
+      </c>
+      <c r="D176" t="inlineStr">
+        <is>
+          <t>TOP</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>BRCB</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>XZO</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>BYND</t>
+        </is>
+      </c>
+      <c r="D177" t="inlineStr">
+        <is>
           <t>USDEW</t>
         </is>
       </c>
-      <c r="C161" t="inlineStr">
-        <is>
-          <t>FIGR</t>
-        </is>
-      </c>
-      <c r="D161" t="inlineStr">
-        <is>
-          <t>NXPL</t>
-        </is>
-      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>SSMR</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>BR</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>SOPH</t>
+        </is>
+      </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>OABI</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>OTLY</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>PRQR</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>MINE</t>
+        </is>
+      </c>
+      <c r="D179" t="inlineStr">
+        <is>
+          <t>DCBO</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>PFX</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>ACOG</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>SAIH</t>
+        </is>
+      </c>
+      <c r="D180" t="inlineStr">
+        <is>
+          <t>CETY</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>FBLG</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>HQI</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>CTNM</t>
+        </is>
+      </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>YDES</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>SNDL</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>CGC</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>STKE</t>
+        </is>
+      </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>ABOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>DSC</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>AIFA</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr"/>
+      <c r="D183" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>